<commit_message>
Add Section 8 parameters from Contact Us Forms
Compared Contact Us Forms.xlsx against the baseline and added 41 new
fields under '8 - Additional Activity Information' for Offers - Contact Us.

Excluded 26 form columns already covered in existing baseline sections
(contact identity, account identity, compliance, legacy/future tracking).

New fields include enquiry classification, Eloqua system metadata, media
tracking parameters, authentication flags, and additional UTM/tracking
fields not previously documented.

Attribution, Operational Reporting, Lead Scoring, and Seller Enablement
columns use 'Potential' where the data may support those use cases.
Amanda Reviewed column left blank per request.

Co-authored-by: demodolly <demodolly@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Baseline Data Use Case Alignment - Offers V1.xlsx
+++ b/Baseline Data Use Case Alignment - Offers V1.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V301"/>
+  <dimension ref="A1:V342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="10.73046875" bestFit="1" customWidth="1" style="13" min="1" max="1"/>
@@ -25109,6 +25109,3161 @@
         </is>
       </c>
     </row>
+    <row r="302">
+      <c r="A302" t="n">
+        <v>301</v>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>Eloqua Record ID</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>What is the Eloqua record identifier for this form submission?</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>System-generated Eloqua record identifier assigned at form submission.</t>
+        </is>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>Provides the durable submission identifier for auditability, deduplication, and downstream integrations.</t>
+        </is>
+      </c>
+      <c r="P302" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="n">
+        <v>302</v>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>Date Submitted</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>When was this form submission received?</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>System timestamp captured at form submission.</t>
+        </is>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>Date/Time</t>
+        </is>
+      </c>
+      <c r="M303" t="inlineStr">
+        <is>
+          <t>Supports submission timing, SLA monitoring, and operational reporting.</t>
+        </is>
+      </c>
+      <c r="P303" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="n">
+        <v>303</v>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>Cisco ID Account Creation Opt-In</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>Does the contact want to create a free Cisco ID account?</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>Customer Input</t>
+        </is>
+      </c>
+      <c r="K304" t="inlineStr">
+        <is>
+          <t>Optional checkbox selected by the customer during form submission.</t>
+        </is>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>Checkbox</t>
+        </is>
+      </c>
+      <c r="M304" t="inlineStr">
+        <is>
+          <t>Captures account-creation intent for onboarding, follow-up routing, and experience personalization.</t>
+        </is>
+      </c>
+      <c r="P304" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="Q304" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="R304" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="n">
+        <v>304</v>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>Preferred Language</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>What is the contact's preferred language?</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>Customer Input</t>
+        </is>
+      </c>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>Optional customer-selected language preference captured on the form.</t>
+        </is>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>Picklist/Text</t>
+        </is>
+      </c>
+      <c r="M305" t="inlineStr">
+        <is>
+          <t>Supports localized follow-up, routing, and customer experience personalization.</t>
+        </is>
+      </c>
+      <c r="P305" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="Q305" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="R305" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="n">
+        <v>305</v>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>Enquiry Type</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>What type of enquiry is the contact submitting?</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>Customer Input</t>
+        </is>
+      </c>
+      <c r="K306" t="inlineStr">
+        <is>
+          <t>Required customer-selected enquiry category captured on the Contact Us form.</t>
+        </is>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>Picklist</t>
+        </is>
+      </c>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>Classifies the contact's intent for routing, lead scoring, seller enablement, and operational reporting.</t>
+        </is>
+      </c>
+      <c r="O306" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P306" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="Q306" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="R306" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="n">
+        <v>306</v>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>IRM Enquiry 2</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>What is the secondary IRM enquiry classification?</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>Customer Input</t>
+        </is>
+      </c>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>Optional secondary enquiry classification field captured on the Contact Us form.</t>
+        </is>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>Picklist/Text</t>
+        </is>
+      </c>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>Provides supplemental enquiry classification for routing, scoring, and follow-up context.</t>
+        </is>
+      </c>
+      <c r="P307" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="Q307" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="R307" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="n">
+        <v>307</v>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>Additional Enquiry Details</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>What additional details did the contact provide about their enquiry?</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>Customer Input</t>
+        </is>
+      </c>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>Optional free-text response captured from the customer on the Contact Us form.</t>
+        </is>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>Provides qualitative enquiry context for seller enablement and operational review.</t>
+        </is>
+      </c>
+      <c r="P308" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="Q308" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="R308" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="n">
+        <v>308</v>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>Contact Request</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>Did the contact request follow-up?</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>System-defaulted or derived contact-request flag for Contact Us submissions.</t>
+        </is>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>Indicates follow-up intent for routing, seller enablement, and operational reporting.</t>
+        </is>
+      </c>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P309" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="Q309" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="R309" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="n">
+        <v>309</v>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>ELQ Site ID</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>What is the Eloqua site identifier for this submission?</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>System-captured Eloqua site identifier associated with the form submission.</t>
+        </is>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>Supports site-level operational reporting, validation, and downstream integrations.</t>
+        </is>
+      </c>
+      <c r="P310" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="n">
+        <v>310</v>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>System Updated By</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>Which system process last updated this record?</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>System-captured process name indicating how the record was created or updated.</t>
+        </is>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M311" t="inlineStr">
+        <is>
+          <t>Supports auditability and operational validation of submission source.</t>
+        </is>
+      </c>
+      <c r="P311" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="n">
+        <v>311</v>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>ELQ Form ID</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>What is the Eloqua form identifier for this submission?</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>System-captured Eloqua form identifier for the Contact Us form.</t>
+        </is>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M312" t="inlineStr">
+        <is>
+          <t>Connects the submission to the source form for operational reporting and validation.</t>
+        </is>
+      </c>
+      <c r="O312" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P312" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="n">
+        <v>312</v>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>ELQ Landing Page ID</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>What is the Eloqua landing page identifier for this submission?</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>System-captured Eloqua landing page identifier associated with the submission.</t>
+        </is>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M313" t="inlineStr">
+        <is>
+          <t>Connects the submission to the originating landing page for attribution and operational reporting.</t>
+        </is>
+      </c>
+      <c r="O313" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P313" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="R313" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="n">
+        <v>313</v>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>Form Submit Date</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>What is the form submit date captured by the system?</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>System-captured form submission date passed from Eloqua or Tealium.</t>
+        </is>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>Date/Time</t>
+        </is>
+      </c>
+      <c r="M314" t="inlineStr">
+        <is>
+          <t>Supports submission timing analysis and operational reporting.</t>
+        </is>
+      </c>
+      <c r="P314" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="n">
+        <v>314</v>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>Landing Page ID/URL</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>What landing page did the contact submit the form from?</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool/Tealium</t>
+        </is>
+      </c>
+      <c r="K315" t="inlineStr">
+        <is>
+          <t>Captured from the landing page URL or ID at form submission and passed to Marketing Automation Tool.</t>
+        </is>
+      </c>
+      <c r="L315" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M315" t="inlineStr">
+        <is>
+          <t>Captures landing page context for attribution, operational reporting, and seller enablement.</t>
+        </is>
+      </c>
+      <c r="O315" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P315" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="R315" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="n">
+        <v>315</v>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>Sub Category</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>What is the submission sub-category?</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K316" t="inlineStr">
+        <is>
+          <t>System-assigned sub-category for Contact Us submissions (e.g., Call ASAP).</t>
+        </is>
+      </c>
+      <c r="L316" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M316" t="inlineStr">
+        <is>
+          <t>Supports urgency-based routing, lead scoring, and operational reporting.</t>
+        </is>
+      </c>
+      <c r="O316" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P316" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="Q316" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="R316" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="n">
+        <v>316</v>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>Org Source</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>What is the organizational source for this submission?</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>System-assigned organizational source (e.g., Marketing, CX, IOT) for the submission.</t>
+        </is>
+      </c>
+      <c r="L317" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M317" t="inlineStr">
+        <is>
+          <t>Supports source-based routing, attribution alignment, and operational reporting.</t>
+        </is>
+      </c>
+      <c r="O317" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P317" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="Q317" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="R317" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="n">
+        <v>317</v>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>Contact Flag</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>What is the contact requirement flag for this submission?</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K318" t="inlineStr">
+        <is>
+          <t>System-assigned flag indicating contact requirement status for the submission.</t>
+        </is>
+      </c>
+      <c r="L318" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M318" t="inlineStr">
+        <is>
+          <t>Supports routing validation and operational reporting.</t>
+        </is>
+      </c>
+      <c r="P318" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="n">
+        <v>318</v>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>Common Campaign ID</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>What is the common campaign identifier for this submission?</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool/Tealium</t>
+        </is>
+      </c>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>Captured from campaign tracking parameters and passed to Marketing Automation Tool.</t>
+        </is>
+      </c>
+      <c r="L319" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M319" t="inlineStr">
+        <is>
+          <t>Connects the submission to campaign taxonomy for attribution and operational reporting.</t>
+        </is>
+      </c>
+      <c r="O319" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P319" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="Q319" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="n">
+        <v>319</v>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>Eloqua Campaign ID</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>What is the Eloqua campaign identifier for this submission?</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K320" t="inlineStr">
+        <is>
+          <t>System-captured Eloqua campaign identifier associated with the form submission.</t>
+        </is>
+      </c>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M320" t="inlineStr">
+        <is>
+          <t>Connects the submission to Eloqua campaign reporting and attribution analysis.</t>
+        </is>
+      </c>
+      <c r="O320" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P320" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="n">
+        <v>320</v>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>Event ID</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>What is the event identifier associated with this submission?</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool/Tealium</t>
+        </is>
+      </c>
+      <c r="K321" t="inlineStr">
+        <is>
+          <t>Captured from event tracking parameters and passed to Marketing Automation Tool.</t>
+        </is>
+      </c>
+      <c r="L321" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M321" t="inlineStr">
+        <is>
+          <t>Connects the submission to event-based attribution and operational reporting.</t>
+        </is>
+      </c>
+      <c r="O321" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P321" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="Q321" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="n">
+        <v>321</v>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>What is the form language/locale for this submission?</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K322" t="inlineStr">
+        <is>
+          <t>System-captured locale code (e.g., en_us, ja_jp) for the form submission.</t>
+        </is>
+      </c>
+      <c r="L322" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M322" t="inlineStr">
+        <is>
+          <t>Supports localized operational reporting, routing, and customer experience alignment.</t>
+        </is>
+      </c>
+      <c r="P322" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="Q322" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="R322" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="n">
+        <v>322</v>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>Previous Referrer</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>What was the previous referrer URL before form submission?</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool/Tealium</t>
+        </is>
+      </c>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>Captured by Tealium from the customer's previous referrer and passed to Marketing Automation Tool.</t>
+        </is>
+      </c>
+      <c r="L323" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M323" t="inlineStr">
+        <is>
+          <t>Supports referrer-based attribution journey analysis and operational reporting.</t>
+        </is>
+      </c>
+      <c r="O323" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P323" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="n">
+        <v>323</v>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>CP_GUTC</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>What is the Cisco tracking cookie value for this submission?</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool/Tealium</t>
+        </is>
+      </c>
+      <c r="K324" t="inlineStr">
+        <is>
+          <t>Captured by Tealium tracking cookie and passed to Marketing Automation Tool.</t>
+        </is>
+      </c>
+      <c r="L324" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M324" t="inlineStr">
+        <is>
+          <t>Supports visitor tracking, identity stitching, and attribution analysis.</t>
+        </is>
+      </c>
+      <c r="O324" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P324" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="n">
+        <v>324</v>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>Google Click ID</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>What is the Google click identifier (gclid) for this submission?</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool/Tealium</t>
+        </is>
+      </c>
+      <c r="K325" t="inlineStr">
+        <is>
+          <t>Captured from Google Ads click tracking parameters and passed to Marketing Automation Tool.</t>
+        </is>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M325" t="inlineStr">
+        <is>
+          <t>Supports paid search click-level attribution and campaign performance reporting.</t>
+        </is>
+      </c>
+      <c r="O325" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P325" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="n">
+        <v>325</v>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>Media Campaign Name</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>What is the media campaign name for this submission?</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool/Tealium</t>
+        </is>
+      </c>
+      <c r="K326" t="inlineStr">
+        <is>
+          <t>Captured from media tracking parameters and passed to Marketing Automation Tool.</t>
+        </is>
+      </c>
+      <c r="L326" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M326" t="inlineStr">
+        <is>
+          <t>Supports media campaign attribution and operational reporting.</t>
+        </is>
+      </c>
+      <c r="O326" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P326" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="n">
+        <v>326</v>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>Media Search Keywords</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>What media search keywords are associated with this submission?</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool/Tealium</t>
+        </is>
+      </c>
+      <c r="K327" t="inlineStr">
+        <is>
+          <t>Captured from media search tracking parameters and passed to Marketing Automation Tool.</t>
+        </is>
+      </c>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M327" t="inlineStr">
+        <is>
+          <t>Supports keyword-level attribution analysis and operational reporting.</t>
+        </is>
+      </c>
+      <c r="O327" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P327" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="Q327" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="n">
+        <v>327</v>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>Media Country Site</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>What media country site is associated with this submission?</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool/Tealium</t>
+        </is>
+      </c>
+      <c r="K328" t="inlineStr">
+        <is>
+          <t>Captured from media tracking parameters and passed to Marketing Automation Tool.</t>
+        </is>
+      </c>
+      <c r="L328" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M328" t="inlineStr">
+        <is>
+          <t>Supports geo-based media attribution and operational reporting.</t>
+        </is>
+      </c>
+      <c r="O328" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P328" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="n">
+        <v>328</v>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>Media Creative</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>What media creative is associated with this submission?</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool/Tealium</t>
+        </is>
+      </c>
+      <c r="K329" t="inlineStr">
+        <is>
+          <t>Captured from media creative tracking parameters and passed to Marketing Automation Tool.</t>
+        </is>
+      </c>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M329" t="inlineStr">
+        <is>
+          <t>Supports creative-level attribution and operational reporting.</t>
+        </is>
+      </c>
+      <c r="O329" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P329" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="n">
+        <v>329</v>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>Media Position</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>What media position is associated with this submission?</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool/Tealium</t>
+        </is>
+      </c>
+      <c r="K330" t="inlineStr">
+        <is>
+          <t>Captured from media placement tracking parameters and passed to Marketing Automation Tool.</t>
+        </is>
+      </c>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M330" t="inlineStr">
+        <is>
+          <t>Supports placement position attribution and operational reporting.</t>
+        </is>
+      </c>
+      <c r="O330" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P330" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="n">
+        <v>330</v>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>Media Placement</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>What media placement is associated with this submission?</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool/Tealium</t>
+        </is>
+      </c>
+      <c r="K331" t="inlineStr">
+        <is>
+          <t>Captured from media placement tracking parameters and passed to Marketing Automation Tool.</t>
+        </is>
+      </c>
+      <c r="L331" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M331" t="inlineStr">
+        <is>
+          <t>Supports placement-level attribution and operational reporting.</t>
+        </is>
+      </c>
+      <c r="O331" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P331" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="n">
+        <v>331</v>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>Media Referring Site</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>What media referring site is associated with this submission?</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool/Tealium</t>
+        </is>
+      </c>
+      <c r="K332" t="inlineStr">
+        <is>
+          <t>Captured from media referrer tracking parameters and passed to Marketing Automation Tool.</t>
+        </is>
+      </c>
+      <c r="L332" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M332" t="inlineStr">
+        <is>
+          <t>Supports referrer-based media attribution and operational reporting.</t>
+        </is>
+      </c>
+      <c r="O332" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P332" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="n">
+        <v>332</v>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>Media Unpaid Search</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>What unpaid search media data is associated with this submission?</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool/Tealium</t>
+        </is>
+      </c>
+      <c r="K333" t="inlineStr">
+        <is>
+          <t>Captured from unpaid search media tracking parameters and passed to Marketing Automation Tool.</t>
+        </is>
+      </c>
+      <c r="L333" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M333" t="inlineStr">
+        <is>
+          <t>Supports organic/unpaid search attribution and operational reporting.</t>
+        </is>
+      </c>
+      <c r="O333" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P333" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="n">
+        <v>333</v>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>utm_id</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>What is the UTM ID for this submission?</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool/Tealium</t>
+        </is>
+      </c>
+      <c r="K334" t="inlineStr">
+        <is>
+          <t>Captured by Tealium from the customer's driving URL and passed to Marketing Automation Tool.</t>
+        </is>
+      </c>
+      <c r="L334" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M334" t="inlineStr">
+        <is>
+          <t>Identifies the campaign ID for future attribution, operational, and funnel reporting.</t>
+        </is>
+      </c>
+      <c r="O334" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P334" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="n">
+        <v>334</v>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>Content Asset ID</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>What is the content asset identifier for this submission?</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool/Tealium</t>
+        </is>
+      </c>
+      <c r="K335" t="inlineStr">
+        <is>
+          <t>Captured from content asset tracking parameters and passed to Marketing Automation Tool.</t>
+        </is>
+      </c>
+      <c r="L335" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M335" t="inlineStr">
+        <is>
+          <t>Connects the submission to content assets for attribution and operational reporting.</t>
+        </is>
+      </c>
+      <c r="O335" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P335" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="n">
+        <v>335</v>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>API Validation Error</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>Were any API validation errors captured for this submission?</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K336" t="inlineStr">
+        <is>
+          <t>System-captured API validation error message, if any, during form processing.</t>
+        </is>
+      </c>
+      <c r="L336" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M336" t="inlineStr">
+        <is>
+          <t>Supports operational monitoring, error tracking, and submission quality review.</t>
+        </is>
+      </c>
+      <c r="P336" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="n">
+        <v>336</v>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>Tray Token</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>What is the Tray.io landing page token for this submission?</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool/Tealium</t>
+        </is>
+      </c>
+      <c r="K337" t="inlineStr">
+        <is>
+          <t>Captured landing page token passed from Tealium/Tray.io to Marketing Automation Tool.</t>
+        </is>
+      </c>
+      <c r="L337" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M337" t="inlineStr">
+        <is>
+          <t>Supports landing page validation, orchestration traceability, and operational reporting.</t>
+        </is>
+      </c>
+      <c r="P337" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="n">
+        <v>337</v>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>Redirect to Intersight Login Page</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>Was the contact redirected to the Intersight login page?</t>
+        </is>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K338" t="inlineStr">
+        <is>
+          <t>System flag indicating redirect to Intersight login page during form flow.</t>
+        </is>
+      </c>
+      <c r="L338" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M338" t="inlineStr">
+        <is>
+          <t>Captures login redirect context for routing and follow-up personalization.</t>
+        </is>
+      </c>
+      <c r="P338" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="Q338" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="R338" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="n">
+        <v>338</v>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>Login Flag</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>Was the contact logged in at the time of submission?</t>
+        </is>
+      </c>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K339" t="inlineStr">
+        <is>
+          <t>System-captured flag indicating whether the contact was authenticated at submission.</t>
+        </is>
+      </c>
+      <c r="L339" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M339" t="inlineStr">
+        <is>
+          <t>Supports identity-aware routing, lead scoring, and seller enablement context.</t>
+        </is>
+      </c>
+      <c r="O339" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P339" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="Q339" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="R339" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="n">
+        <v>339</v>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>OKTA Response</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>What OKTA authentication response was captured for this submission?</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K340" t="inlineStr">
+        <is>
+          <t>System-captured OKTA authentication response during login flow, if applicable.</t>
+        </is>
+      </c>
+      <c r="L340" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M340" t="inlineStr">
+        <is>
+          <t>Supports authentication validation and operational troubleshooting.</t>
+        </is>
+      </c>
+      <c r="P340" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="R340" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="n">
+        <v>340</v>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>Contact Source Original</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>What is the original contact source for this submission?</t>
+        </is>
+      </c>
+      <c r="J341" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K341" t="inlineStr">
+        <is>
+          <t>System-captured original source identifier (e.g., Eloqua-Form-submit-ContactSales6493).</t>
+        </is>
+      </c>
+      <c r="L341" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M341" t="inlineStr">
+        <is>
+          <t>Supports source lineage for attribution, operational reporting, and seller enablement.</t>
+        </is>
+      </c>
+      <c r="O341" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P341" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="R341" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="n">
+        <v>341</v>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Online Forms</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Hand Raiser</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Offers - Contact Us</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Form Submit</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>8 - Additional Activity Information</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>Contact Sales</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>Did the contact request sales contact?</t>
+        </is>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>Marketing Automation Tool</t>
+        </is>
+      </c>
+      <c r="K342" t="inlineStr">
+        <is>
+          <t>System-captured contact sales flag for the submission.</t>
+        </is>
+      </c>
+      <c r="L342" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="M342" t="inlineStr">
+        <is>
+          <t>Supports sales routing, lead scoring, and seller enablement decisions.</t>
+        </is>
+      </c>
+      <c r="O342" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="P342" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="Q342" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="R342" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V206"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>